<commit_message>
v15 colour-LCD board, firmware with live preview, CAD and docs
- v14 frozen (tag v14-order, archive copies)
- v15-LCD PCB: 1.9in ST7789 IPS (BuyDisplay ER-TFT019-1), J5 mirrored,
  slot/J5 moved for the tail bow, R23 15 ohm, SHIFT/ALPHA/ON pads matched
  to the Casio board; reviews 13-15 verdict ORDER; fab_v15_lcd outputs
- firmware-v15-lcd: LovyanGFX colour UI, backlight, live camera preview
- OTA server: never offers one board family's image to the other
- CAD v15 fit model, v15 assembly and power-up guides, order walkthrough
- Budget, cost model, roadmap and status docs updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Claude outputs/Alibaba_Bulk_Sourcing.xlsx
+++ b/Claude outputs/Alibaba_Bulk_Sourcing.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="Cost by batch" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Supplier options" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Supplier message templates" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Checks before bulk" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sources" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="v15-LCD cost by batch" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Supplier options" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Supplier message templates" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Checks before bulk" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sources" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Supplier options'!$A$3:$L$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Supplier options'!$A$3:$L$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,6 +77,11 @@
       <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -121,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -170,6 +176,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2120,7 +2143,1984 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:R49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="60" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>AI Calculator v15-LCD: bulk cost per unit at 10 / 100 / 1,000 units (1.9" colour LCD instead of the e-paper; knockoff 991ES-style shell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Added 2026-10-08, updated 2026-10-08 evening. Same layout as 'Cost by batch'; every row links to it except row 1 (PCBA + v15 change) and row 4 (LCD panel). Blue = inputs. v15 board verified 'ORDER' (hardware/verification/14_v15_final_preorder.md); upload files hardware/fab_v15_lcd/, steps hardware/ORDER_WALKTHROUGH_v15_lcd.md. Panel: BuyDisplay ER-TFT019-1 (datasheet-verified). Bigger battery option below the total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Batch size →</t>
+        </is>
+      </c>
+      <c r="O3" s="25">
+        <f>'Cost by batch'!O3</f>
+        <v/>
+      </c>
+      <c r="P3" s="25">
+        <f>'Cost by batch'!P3</f>
+        <v/>
+      </c>
+      <c r="Q3" s="25">
+        <f>'Cost by batch'!Q3</f>
+        <v/>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>← batch sizes come from 'Cost by batch'</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Item &amp; key spec</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Source @10</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Source @100</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Source @1,000</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Main link</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Qty / unit</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Unit $ @10</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>Unit $ @100</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>Unit $ @1,000</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Per-unit $ @10</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>Per-unit $ @100</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>Per-unit $ @1,000</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>Batch total @10</t>
+        </is>
+      </c>
+      <c r="P4" s="6" t="inlineStr">
+        <is>
+          <t>Batch total @100</t>
+        </is>
+      </c>
+      <c r="Q4" s="6" t="inlineStr">
+        <is>
+          <t>Batch total @1,000</t>
+        </is>
+      </c>
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>Price basis / notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>PCBA</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Main board v15-LCD: PCB 2-layer 0.8 mm ENIG + Standard PCBA (v14 board minus the e-paper booster, plus J5 30-pin socket, Q4/Q5 LCD power + backlight FETs, R23 15 Ω C22810)</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>JLCPCB (Economic/Standard PCBA)</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="14">
+        <f>'Cost by batch'!I5+$I$35-$I$36+$I$37*$I$38/O$3</f>
+        <v/>
+      </c>
+      <c r="J5" s="14">
+        <f>'Cost by batch'!J5+$I$35-$I$36+$I$37*$I$38/P$3</f>
+        <v/>
+      </c>
+      <c r="K5" s="14">
+        <f>'Cost by batch'!K5+$I$35-$I$36+$I$37*$I$38/Q$3</f>
+        <v/>
+      </c>
+      <c r="L5" s="11">
+        <f>$H5*I5</f>
+        <v/>
+      </c>
+      <c r="M5" s="11">
+        <f>$H5*J5</f>
+        <v/>
+      </c>
+      <c r="N5" s="11">
+        <f>$H5*K5</f>
+        <v/>
+      </c>
+      <c r="O5" s="11">
+        <f>L5*O$3</f>
+        <v/>
+      </c>
+      <c r="P5" s="11">
+        <f>M5*P$3</f>
+        <v/>
+      </c>
+      <c r="Q5" s="11">
+        <f>N5*Q$3</f>
+        <v/>
+      </c>
+      <c r="R5" s="12" t="inlineStr">
+        <is>
+          <t>'Cost by batch' PCBA price + (parts added − removed) + extended-type change × $3 ÷ batch. Files: hardware/fab_v15_lcd/ (21:38). Verified ORDER (review 14), not yet ordered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Knockoff 991ES PLUS-style calculator (shell, key mat, window, screws, slide cover); board removed</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>AliExpress / Amazon (MOQ 1)</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba (MOQ ~20-50)</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba factory (same mould, MOQ 500-3,000)</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H6" s="7">
+        <f>'Cost by batch'!H6</f>
+        <v/>
+      </c>
+      <c r="I6" s="14">
+        <f>'Cost by batch'!I6</f>
+        <v/>
+      </c>
+      <c r="J6" s="14">
+        <f>'Cost by batch'!J6</f>
+        <v/>
+      </c>
+      <c r="K6" s="14">
+        <f>'Cost by batch'!K6</f>
+        <v/>
+      </c>
+      <c r="L6" s="11">
+        <f>$H6*I6</f>
+        <v/>
+      </c>
+      <c r="M6" s="11">
+        <f>$H6*J6</f>
+        <v/>
+      </c>
+      <c r="N6" s="11">
+        <f>$H6*K6</f>
+        <v/>
+      </c>
+      <c r="O6" s="11">
+        <f>L6*O$3</f>
+        <v/>
+      </c>
+      <c r="P6" s="11">
+        <f>M6*P$3</f>
+        <v/>
+      </c>
+      <c r="Q6" s="11">
+        <f>N6*Q$3</f>
+        <v/>
+      </c>
+      <c r="R6" s="12" t="inlineStr">
+        <is>
+          <t>Alibaba listing seen at $3.25-3.99, MOQ 20 [S1]; factories quote $1.50-3.50 at MOQ 3,000 [S2]. @10 = retail clone incl. shipping (estimate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>OV5640 AF, 24-pin 0.5 mm FPC DVP, Seeed XIAO-Sense pinout, AF lens</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Seeed SS114993115 (known pinout)</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba OEM (V-Vision etc.) after pinout check</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba OEM, custom FPC length</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H7" s="7">
+        <f>'Cost by batch'!H7</f>
+        <v/>
+      </c>
+      <c r="I7" s="14">
+        <f>'Cost by batch'!I7</f>
+        <v/>
+      </c>
+      <c r="J7" s="14">
+        <f>'Cost by batch'!J7</f>
+        <v/>
+      </c>
+      <c r="K7" s="14">
+        <f>'Cost by batch'!K7</f>
+        <v/>
+      </c>
+      <c r="L7" s="11">
+        <f>$H7*I7</f>
+        <v/>
+      </c>
+      <c r="M7" s="11">
+        <f>$H7*J7</f>
+        <v/>
+      </c>
+      <c r="N7" s="11">
+        <f>$H7*K7</f>
+        <v/>
+      </c>
+      <c r="O7" s="11">
+        <f>L7*O$3</f>
+        <v/>
+      </c>
+      <c r="P7" s="11">
+        <f>M7*P$3</f>
+        <v/>
+      </c>
+      <c r="Q7" s="11">
+        <f>N7*Q$3</f>
+        <v/>
+      </c>
+      <c r="R7" s="12" t="inlineStr">
+        <is>
+          <t>Roadmap table [S8]; Alibaba OV5640 24-pin modules ~$5-18 [S3]; eBay/AliExpress AF 24-pin ~GBP 7.49 [S4].</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>1.9" 170×320 IPS LCD, ST7789, 30-pin 0.5 mm FPC (36.6 mm tail), 4 white LEDs; TFT1901 / N190-1732TBWPG01 family (LilyGO T-Display-S3 panel)</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>BuyDisplay ER-TFT019-1, no touch (datasheet-verified pin for pin)</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba Goldenmorning T190X7-C30-01 / ZJY, after a sample check</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba / panel maker; optional short-tail FPC (Goldenmorning, TSD, NoseDisplay, BuyDisplay custom FPC)</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="14">
+        <f>$I$31+$I$32/O$3</f>
+        <v/>
+      </c>
+      <c r="J8" s="14">
+        <f>$I$33</f>
+        <v/>
+      </c>
+      <c r="K8" s="14">
+        <f>$I$34</f>
+        <v/>
+      </c>
+      <c r="L8" s="11">
+        <f>$H8*I8</f>
+        <v/>
+      </c>
+      <c r="M8" s="11">
+        <f>$H8*J8</f>
+        <v/>
+      </c>
+      <c r="N8" s="11">
+        <f>$H8*K8</f>
+        <v/>
+      </c>
+      <c r="O8" s="11">
+        <f>L8*O$3</f>
+        <v/>
+      </c>
+      <c r="P8" s="11">
+        <f>M8*P$3</f>
+        <v/>
+      </c>
+      <c r="Q8" s="11">
+        <f>N8*Q$3</f>
+        <v/>
+      </c>
+      <c r="R8" s="12" t="inlineStr">
+        <is>
+          <t>@10: BuyDisplay ER-TFT019-1 $6.22 each @10 ($5.71 @100) + one shipping charge shared by the batch (estimate). @100/@1,000: Alibaba ZJY (Zhengzhou Zhongjingyuan) ST7789V3 30-pin $2.50 @100 / $2.30 @1,000, MOQ 2, or Goldenmorning T190X7-C30-01 (plastic frame) (hardware/production/lcd_suppliers.json; search-snippet prices, confirm by quote and a sample check) [S15]. Adafruit #5394 ($17.50) is only an optional fallback now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>LiPo 3.7 V ~150 mAh with PCM, JST-PH 2.0 plug (red = +, Adafruit polarity), Adafruit #1317 class 26 × 19.75 × 3.8 mm; max 33.5 × 20.7 × 3.8 mm incl. PCM fold</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Adafruit #1317</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba stock cell + PH2.0 lead</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba custom cell (~382026 / 402025 class, 150 mAh) with certs</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H9" s="7">
+        <f>'Cost by batch'!H9</f>
+        <v/>
+      </c>
+      <c r="I9" s="14">
+        <f>'Cost by batch'!I9</f>
+        <v/>
+      </c>
+      <c r="J9" s="14">
+        <f>'Cost by batch'!J9</f>
+        <v/>
+      </c>
+      <c r="K9" s="14">
+        <f>'Cost by batch'!K9</f>
+        <v/>
+      </c>
+      <c r="L9" s="11">
+        <f>$H9*I9</f>
+        <v/>
+      </c>
+      <c r="M9" s="11">
+        <f>$H9*J9</f>
+        <v/>
+      </c>
+      <c r="N9" s="11">
+        <f>$H9*K9</f>
+        <v/>
+      </c>
+      <c r="O9" s="11">
+        <f>L9*O$3</f>
+        <v/>
+      </c>
+      <c r="P9" s="11">
+        <f>M9*P$3</f>
+        <v/>
+      </c>
+      <c r="Q9" s="11">
+        <f>N9*Q$3</f>
+        <v/>
+      </c>
+      <c r="R9" s="12" t="inlineStr">
+        <is>
+          <t>Adafruit #1317 $5.95 [S8] (switched from the 100 mAh #1570 on 2026-10-06; same price). Alibaba 401230 listings $0.56-1.60 [S6] are 100 mAh references (401230 is 4.0 x 12 x 30: too thick and wide); ask for a ~150 mAh cell in 26 x 20 x 3.8. @100/@1,000 include PH lead + PCM (estimate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Dangerous-goods (UN3481) air-freight surcharge for batteries, per unit</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>(in Adafruit price)</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba supplier DG air / express</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Sea or DG air with the cells</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7">
+        <f>'Cost by batch'!H10</f>
+        <v/>
+      </c>
+      <c r="I10" s="14">
+        <f>'Cost by batch'!I10</f>
+        <v/>
+      </c>
+      <c r="J10" s="14">
+        <f>'Cost by batch'!J10</f>
+        <v/>
+      </c>
+      <c r="K10" s="14">
+        <f>'Cost by batch'!K10</f>
+        <v/>
+      </c>
+      <c r="L10" s="11">
+        <f>$H10*I10</f>
+        <v/>
+      </c>
+      <c r="M10" s="11">
+        <f>$H10*J10</f>
+        <v/>
+      </c>
+      <c r="N10" s="11">
+        <f>$H10*K10</f>
+        <v/>
+      </c>
+      <c r="O10" s="11">
+        <f>L10*O$3</f>
+        <v/>
+      </c>
+      <c r="P10" s="11">
+        <f>M10*P$3</f>
+        <v/>
+      </c>
+      <c r="Q10" s="11">
+        <f>N10*Q$3</f>
+        <v/>
+      </c>
+      <c r="R10" s="12" t="inlineStr">
+        <is>
+          <t>Estimate. Many forwarders refuse loose LiPo; ask the supplier to ship with UN38.3 + MSDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Charging</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>4-pin magnetic pogo connector pair, ~2.54 mm pitch, board half fits J3 (VBUS, D-, D+, GND from N end)</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Adafruit #5358</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba RA pogo pair (sample-checked)</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba OEM pair, drawing-approved</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H11" s="7">
+        <f>'Cost by batch'!H11</f>
+        <v/>
+      </c>
+      <c r="I11" s="14">
+        <f>'Cost by batch'!I11</f>
+        <v/>
+      </c>
+      <c r="J11" s="14">
+        <f>'Cost by batch'!J11</f>
+        <v/>
+      </c>
+      <c r="K11" s="14">
+        <f>'Cost by batch'!K11</f>
+        <v/>
+      </c>
+      <c r="L11" s="11">
+        <f>$H11*I11</f>
+        <v/>
+      </c>
+      <c r="M11" s="11">
+        <f>$H11*J11</f>
+        <v/>
+      </c>
+      <c r="N11" s="11">
+        <f>$H11*K11</f>
+        <v/>
+      </c>
+      <c r="O11" s="11">
+        <f>L11*O$3</f>
+        <v/>
+      </c>
+      <c r="P11" s="11">
+        <f>M11*P$3</f>
+        <v/>
+      </c>
+      <c r="Q11" s="11">
+        <f>N11*Q$3</f>
+        <v/>
+      </c>
+      <c r="R11" s="12" t="inlineStr">
+        <is>
+          <t>Adafruit $5.85 @10 [S8]; Alibaba MG04-254-RA $1.80, multiples of 20 [S7]; roadmap $1.20 @1,000 (estimate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Charging</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Magnetic USB cable for the 4-pin connector (cable N-&gt;S: GND, D+, D-, VBUS), in the box</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Adafruit #5412</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba (same supplier as connector)</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba OEM, same supplier as connector</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H12" s="7">
+        <f>'Cost by batch'!H12</f>
+        <v/>
+      </c>
+      <c r="I12" s="14">
+        <f>'Cost by batch'!I12</f>
+        <v/>
+      </c>
+      <c r="J12" s="14">
+        <f>'Cost by batch'!J12</f>
+        <v/>
+      </c>
+      <c r="K12" s="14">
+        <f>'Cost by batch'!K12</f>
+        <v/>
+      </c>
+      <c r="L12" s="11">
+        <f>$H12*I12</f>
+        <v/>
+      </c>
+      <c r="M12" s="11">
+        <f>$H12*J12</f>
+        <v/>
+      </c>
+      <c r="N12" s="11">
+        <f>$H12*K12</f>
+        <v/>
+      </c>
+      <c r="O12" s="11">
+        <f>L12*O$3</f>
+        <v/>
+      </c>
+      <c r="P12" s="11">
+        <f>M12*P$3</f>
+        <v/>
+      </c>
+      <c r="Q12" s="11">
+        <f>N12*Q$3</f>
+        <v/>
+      </c>
+      <c r="R12" s="12" t="inlineStr">
+        <is>
+          <t>Adafruit $4.95 [S8]; roadmap estimate $1.40-1.80 for OEM cable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Retail box + foam/EVA insert (printed)</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Plain mailer box (local / Amazon)</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba custom rigid box, MOQ 100</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba custom box + die-cut insert</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H13" s="7">
+        <f>'Cost by batch'!H13</f>
+        <v/>
+      </c>
+      <c r="I13" s="14">
+        <f>'Cost by batch'!I13</f>
+        <v/>
+      </c>
+      <c r="J13" s="14">
+        <f>'Cost by batch'!J13</f>
+        <v/>
+      </c>
+      <c r="K13" s="14">
+        <f>'Cost by batch'!K13</f>
+        <v/>
+      </c>
+      <c r="L13" s="11">
+        <f>$H13*I13</f>
+        <v/>
+      </c>
+      <c r="M13" s="11">
+        <f>$H13*J13</f>
+        <v/>
+      </c>
+      <c r="N13" s="11">
+        <f>$H13*K13</f>
+        <v/>
+      </c>
+      <c r="O13" s="11">
+        <f>L13*O$3</f>
+        <v/>
+      </c>
+      <c r="P13" s="11">
+        <f>M13*P$3</f>
+        <v/>
+      </c>
+      <c r="Q13" s="11">
+        <f>N13*Q$3</f>
+        <v/>
+      </c>
+      <c r="R13" s="12" t="inlineStr">
+        <is>
+          <t>Alibaba rigid boxes w/ foam insert $0.50-1.00 at MOQ 100 [S9]; @10 estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Quick-start card / small manual (with 'not affiliated with Casio', FCC text later)</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Home print</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Local / online printer</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba printer (MOQ 500)</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H14" s="7">
+        <f>'Cost by batch'!H14</f>
+        <v/>
+      </c>
+      <c r="I14" s="14">
+        <f>'Cost by batch'!I14</f>
+        <v/>
+      </c>
+      <c r="J14" s="14">
+        <f>'Cost by batch'!J14</f>
+        <v/>
+      </c>
+      <c r="K14" s="14">
+        <f>'Cost by batch'!K14</f>
+        <v/>
+      </c>
+      <c r="L14" s="11">
+        <f>$H14*I14</f>
+        <v/>
+      </c>
+      <c r="M14" s="11">
+        <f>$H14*J14</f>
+        <v/>
+      </c>
+      <c r="N14" s="11">
+        <f>$H14*K14</f>
+        <v/>
+      </c>
+      <c r="O14" s="11">
+        <f>L14*O$3</f>
+        <v/>
+      </c>
+      <c r="P14" s="11">
+        <f>M14*P$3</f>
+        <v/>
+      </c>
+      <c r="Q14" s="11">
+        <f>N14*Q$3</f>
+        <v/>
+      </c>
+      <c r="R14" s="12" t="inlineStr">
+        <is>
+          <t>Manual printing $0.03 (500+) to $0.01 (10k+) [S10]; small runs estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Serial / QC label sticker + polybag for calculator</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Home print</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Online label printer</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba / Uline</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H15" s="7">
+        <f>'Cost by batch'!H15</f>
+        <v/>
+      </c>
+      <c r="I15" s="14">
+        <f>'Cost by batch'!I15</f>
+        <v/>
+      </c>
+      <c r="J15" s="14">
+        <f>'Cost by batch'!J15</f>
+        <v/>
+      </c>
+      <c r="K15" s="14">
+        <f>'Cost by batch'!K15</f>
+        <v/>
+      </c>
+      <c r="L15" s="11">
+        <f>$H15*I15</f>
+        <v/>
+      </c>
+      <c r="M15" s="11">
+        <f>$H15*J15</f>
+        <v/>
+      </c>
+      <c r="N15" s="11">
+        <f>$H15*K15</f>
+        <v/>
+      </c>
+      <c r="O15" s="11">
+        <f>L15*O$3</f>
+        <v/>
+      </c>
+      <c r="P15" s="11">
+        <f>M15*P$3</f>
+        <v/>
+      </c>
+      <c r="Q15" s="11">
+        <f>N15*Q$3</f>
+        <v/>
+      </c>
+      <c r="R15" s="12" t="inlineStr">
+        <is>
+          <t>Estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Consumables</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Kapton tape 10 mm, thin double-sided tape (3M 9448A-type), B-7000/E6000 glue; per unit share</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Amazon / AliExpress</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>AliExpress / LCSC</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba bulk rolls</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H16" s="7">
+        <f>'Cost by batch'!H16</f>
+        <v/>
+      </c>
+      <c r="I16" s="14">
+        <f>'Cost by batch'!I16</f>
+        <v/>
+      </c>
+      <c r="J16" s="14">
+        <f>'Cost by batch'!J16</f>
+        <v/>
+      </c>
+      <c r="K16" s="14">
+        <f>'Cost by batch'!K16</f>
+        <v/>
+      </c>
+      <c r="L16" s="11">
+        <f>$H16*I16</f>
+        <v/>
+      </c>
+      <c r="M16" s="11">
+        <f>$H16*J16</f>
+        <v/>
+      </c>
+      <c r="N16" s="11">
+        <f>$H16*K16</f>
+        <v/>
+      </c>
+      <c r="O16" s="11">
+        <f>L16*O$3</f>
+        <v/>
+      </c>
+      <c r="P16" s="11">
+        <f>M16*P$3</f>
+        <v/>
+      </c>
+      <c r="Q16" s="11">
+        <f>N16*Q$3</f>
+        <v/>
+      </c>
+      <c r="R16" s="12" t="inlineStr">
+        <is>
+          <t>Estimate (a 30 m roll covers roughly 100+ units).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Freight</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Inbound freight + US import duty on China content (PCBA, parts, shells)</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>DHL (JLCPCB DDP)</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>DHL / consolidated</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Forwarder, sea/air LCL</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H17" s="7">
+        <f>'Cost by batch'!H17</f>
+        <v/>
+      </c>
+      <c r="I17" s="14">
+        <f>'Cost by batch'!I17</f>
+        <v/>
+      </c>
+      <c r="J17" s="14">
+        <f>'Cost by batch'!J17</f>
+        <v/>
+      </c>
+      <c r="K17" s="14">
+        <f>'Cost by batch'!K17</f>
+        <v/>
+      </c>
+      <c r="L17" s="11">
+        <f>$H17*I17</f>
+        <v/>
+      </c>
+      <c r="M17" s="11">
+        <f>$H17*J17</f>
+        <v/>
+      </c>
+      <c r="N17" s="11">
+        <f>$H17*K17</f>
+        <v/>
+      </c>
+      <c r="O17" s="11">
+        <f>L17*O$3</f>
+        <v/>
+      </c>
+      <c r="P17" s="11">
+        <f>M17*P$3</f>
+        <v/>
+      </c>
+      <c r="Q17" s="11">
+        <f>N17*Q$3</f>
+        <v/>
+      </c>
+      <c r="R17" s="12" t="inlineStr">
+        <is>
+          <t>Roadmap table, assumes ~35 % duty (low end of 35-92.5 %) [S8]. Biggest swing factor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Final assembly (strip knockoff, mask, grind, fit board, test)</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Nirav</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Nirav (+ jig)</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>EMS box build / local helper</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7">
+        <f>'Cost by batch'!H18</f>
+        <v/>
+      </c>
+      <c r="I18" s="14">
+        <f>'Cost by batch'!I18</f>
+        <v/>
+      </c>
+      <c r="J18" s="14">
+        <f>'Cost by batch'!J18</f>
+        <v/>
+      </c>
+      <c r="K18" s="14">
+        <f>'Cost by batch'!K18</f>
+        <v/>
+      </c>
+      <c r="L18" s="11">
+        <f>$H18*I18</f>
+        <v/>
+      </c>
+      <c r="M18" s="11">
+        <f>$H18*J18</f>
+        <v/>
+      </c>
+      <c r="N18" s="11">
+        <f>$H18*K18</f>
+        <v/>
+      </c>
+      <c r="O18" s="11">
+        <f>L18*O$3</f>
+        <v/>
+      </c>
+      <c r="P18" s="11">
+        <f>M18*P$3</f>
+        <v/>
+      </c>
+      <c r="Q18" s="11">
+        <f>N18*Q$3</f>
+        <v/>
+      </c>
+      <c r="R18" s="12" t="inlineStr">
+        <is>
+          <t>Roadmap table (estimate). Your own time is not costed at 10/100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Overage</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Scrap + spares allowance (% of rows above, excl. labour) — DOA cameras/panels, cracked shells</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Allowance %:</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="26">
+        <f>'Cost by batch'!I19</f>
+        <v/>
+      </c>
+      <c r="J19" s="26">
+        <f>'Cost by batch'!J19</f>
+        <v/>
+      </c>
+      <c r="K19" s="26">
+        <f>'Cost by batch'!K19</f>
+        <v/>
+      </c>
+      <c r="L19" s="14">
+        <f>I19*(SUM(L5:L18)-L18)</f>
+        <v/>
+      </c>
+      <c r="M19" s="14">
+        <f>J19*(SUM(M5:M18)-M18)</f>
+        <v/>
+      </c>
+      <c r="N19" s="14">
+        <f>K19*(SUM(N5:N18)-N18)</f>
+        <v/>
+      </c>
+      <c r="O19" s="14">
+        <f>L19*O$3</f>
+        <v/>
+      </c>
+      <c r="P19" s="14">
+        <f>M19*P$3</f>
+        <v/>
+      </c>
+      <c r="Q19" s="14">
+        <f>N19*Q$3</f>
+        <v/>
+      </c>
+      <c r="R19" s="12" t="inlineStr">
+        <is>
+          <t>Estimate. Order this many extra parts, not just budget for them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>One-time</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Samples from each supplier (2 each, from 2 suppliers per part) + express shipping</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>per batch</t>
+        </is>
+      </c>
+      <c r="I20" s="14">
+        <f>'Cost by batch'!I20</f>
+        <v/>
+      </c>
+      <c r="J20" s="14">
+        <f>'Cost by batch'!J20</f>
+        <v/>
+      </c>
+      <c r="K20" s="14">
+        <f>'Cost by batch'!K20</f>
+        <v/>
+      </c>
+      <c r="L20" s="14">
+        <f>I20/O$3</f>
+        <v/>
+      </c>
+      <c r="M20" s="14">
+        <f>J20/P$3</f>
+        <v/>
+      </c>
+      <c r="N20" s="14">
+        <f>K20/Q$3</f>
+        <v/>
+      </c>
+      <c r="O20" s="14">
+        <f>I20</f>
+        <v/>
+      </c>
+      <c r="P20" s="14">
+        <f>J20</f>
+        <v/>
+      </c>
+      <c r="Q20" s="14">
+        <f>K20</f>
+        <v/>
+      </c>
+      <c r="R20" s="12" t="inlineStr">
+        <is>
+          <t>Estimate. Per-unit = amount / batch size. Repeat a smaller sample round whenever you change supplier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>One-time</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Pre-shipment inspection / golden-sample sign-off (third-party QC, e.g. 1 man-day)</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>per batch</t>
+        </is>
+      </c>
+      <c r="I21" s="14">
+        <f>'Cost by batch'!I21</f>
+        <v/>
+      </c>
+      <c r="J21" s="14">
+        <f>'Cost by batch'!J21</f>
+        <v/>
+      </c>
+      <c r="K21" s="14">
+        <f>'Cost by batch'!K21</f>
+        <v/>
+      </c>
+      <c r="L21" s="14">
+        <f>I21/O$3</f>
+        <v/>
+      </c>
+      <c r="M21" s="14">
+        <f>J21/P$3</f>
+        <v/>
+      </c>
+      <c r="N21" s="14">
+        <f>K21/Q$3</f>
+        <v/>
+      </c>
+      <c r="O21" s="14">
+        <f>I21</f>
+        <v/>
+      </c>
+      <c r="P21" s="14">
+        <f>J21</f>
+        <v/>
+      </c>
+      <c r="Q21" s="14">
+        <f>K21</f>
+        <v/>
+      </c>
+      <c r="R21" s="12" t="inlineStr">
+        <is>
+          <t>Estimate (~$300 per man-day typical). Only worth it at 1,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>One-time</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Test jig (pogo bed + spring pins) and fixtures</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>per batch</t>
+        </is>
+      </c>
+      <c r="I22" s="14">
+        <f>'Cost by batch'!I22</f>
+        <v/>
+      </c>
+      <c r="J22" s="14">
+        <f>'Cost by batch'!J22</f>
+        <v/>
+      </c>
+      <c r="K22" s="14">
+        <f>'Cost by batch'!K22</f>
+        <v/>
+      </c>
+      <c r="L22" s="14">
+        <f>I22/O$3</f>
+        <v/>
+      </c>
+      <c r="M22" s="14">
+        <f>J22/P$3</f>
+        <v/>
+      </c>
+      <c r="N22" s="14">
+        <f>K22/Q$3</f>
+        <v/>
+      </c>
+      <c r="O22" s="14">
+        <f>I22</f>
+        <v/>
+      </c>
+      <c r="P22" s="14">
+        <f>J22</f>
+        <v/>
+      </c>
+      <c r="Q22" s="14">
+        <f>K22</f>
+        <v/>
+      </c>
+      <c r="R22" s="12" t="inlineStr">
+        <is>
+          <t>Roadmap §5 estimate $50-150.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="n"/>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="inlineStr">
+        <is>
+          <t>Per-unit / batch →</t>
+        </is>
+      </c>
+      <c r="L23" s="16">
+        <f>SUM(L5:L22)</f>
+        <v/>
+      </c>
+      <c r="M23" s="16">
+        <f>SUM(M5:M22)</f>
+        <v/>
+      </c>
+      <c r="N23" s="16">
+        <f>SUM(N5:N22)</f>
+        <v/>
+      </c>
+      <c r="O23" s="16">
+        <f>SUM(O5:O22)</f>
+        <v/>
+      </c>
+      <c r="P23" s="16">
+        <f>SUM(P5:P22)</f>
+        <v/>
+      </c>
+      <c r="Q23" s="16">
+        <f>SUM(Q5:Q22)</f>
+        <v/>
+      </c>
+      <c r="R23" s="15" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n"/>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Check: batch total / batch size (should equal the per-unit total)</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="n"/>
+      <c r="H24" s="5" t="n"/>
+      <c r="I24" s="5" t="n"/>
+      <c r="J24" s="5" t="n"/>
+      <c r="K24" s="5" t="n"/>
+      <c r="L24" s="17">
+        <f>O23/O$3</f>
+        <v/>
+      </c>
+      <c r="M24" s="17">
+        <f>P23/P$3</f>
+        <v/>
+      </c>
+      <c r="N24" s="17">
+        <f>Q23/Q$3</f>
+        <v/>
+      </c>
+      <c r="O24" s="5" t="n"/>
+      <c r="P24" s="5" t="n"/>
+      <c r="Q24" s="5" t="n"/>
+      <c r="R24" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Note: LCD vs e-paper: the panel itself is ~$6.22 at 10 (BuyDisplay) and ~$2.30-2.50 at 100+ (Alibaba) instead of $4-6.60, and the board loses 17 booster parts and gains 7. But the LCD draws ~80-90 mA with the screen on: ~1.5 h screen-on on the 150 mAh cell (stage15_lcd.md §3), so the long-term pairing is the 1,200-1,500 mAh cell below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Note: Not included (as on 'Cost by batch'): FCC SDoC, LLC, lawyer, trademark (≈ $3.5k one-time), Claude API, sales fees. Full model: hardware/production/COST_MODEL.xlsx 'Versions'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>Inputs for the LCD version</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="C31" s="27" t="inlineStr">
+        <is>
+          <t>LCD panel @10: BuyDisplay ER-TFT019-1 (no touch), per panel at the 10-pc price</t>
+        </is>
+      </c>
+      <c r="I31" s="28" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>Given 2026-10-08 (review 14 / LCD_PANEL_OPTIONS.md): ~$6-7 each, $6.22 @10, $5.71 @100. Datasheet rev 2.0 checked pin for pin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" s="27" t="inlineStr">
+        <is>
+          <t>BuyDisplay shipping per order (estimate)</t>
+        </is>
+      </c>
+      <c r="I32" s="28" t="n">
+        <v>12</v>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>Estimate, not quoted: check at checkout on buydisplay.com and replace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33" s="27" t="inlineStr">
+        <is>
+          <t>LCD panel @100 (Alibaba / panel maker)</t>
+        </is>
+      </c>
+      <c r="I33" s="28" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>Alibaba ZJY (Zhengzhou Zhongjingyuan) ST7789V3 30-pin $2.50 @100 / $2.30 @1,000, MOQ 2 (hardware/production/lcd_suppliers.json, 2026-10-08; search-snippet prices, confirm by quote) [S15].</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="C34" s="27" t="inlineStr">
+        <is>
+          <t>LCD panel @1,000 (Alibaba / panel maker, maybe short-tail FPC)</t>
+        </is>
+      </c>
+      <c r="I34" s="28" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>Alibaba ZJY (Zhengzhou Zhongjingyuan) ST7789V3 30-pin $2.50 @100 / $2.30 @1,000, MOQ 2 (hardware/production/lcd_suppliers.json, 2026-10-08; search-snippet prices, confirm by quote) [S15]. Ask NoseDisplay / BuyDisplay / QDtech for an 18-20 mm FPC tail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>v15 parts added per board: J5 C2919501 $0.36 + Q4 AO3401A $0.10 + Q5 AO3400A C20917 $0.09 + R21, R22, C36 3 × $0.002 + R23 15 Ω C22810 $0.0013</t>
+        </is>
+      </c>
+      <c r="I35" s="28" t="n">
+        <v>0.5573</v>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>JLCPCB prices 2026-10-08 (stage15_lcd.md §3; R23 changed to 15 Ω C22810 in review 14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="C36" s="27" t="inlineStr">
+        <is>
+          <t>v14 e-paper parts removed per board: J2, L1, Q3, R11, R12, D3-D5, C20-C30 (17 parts)</t>
+        </is>
+      </c>
+      <c r="I36" s="28" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>Estimate from LCSC 1-off prices; stage 15: board ≈ $1 cheaper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="C37" s="27" t="inlineStr">
+        <is>
+          <t>Change in JLCPCB extended part types (L1, Q3, R12 out; J5 C2919501 and R23 C22810 in)</t>
+        </is>
+      </c>
+      <c r="I37" s="29" t="n">
+        <v>-1</v>
+      </c>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>v14 had 14 extended types, v15 has 13 (review 14 stock list). $3 per type per order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="C38" s="27" t="inlineStr">
+        <is>
+          <t>Extended-part fee per type per order</t>
+        </is>
+      </c>
+      <c r="I38" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>JLCPCB rule (roadmap §3.1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="21" t="inlineStr">
+        <is>
+          <t>Compare and bigger-battery option (per unit)</t>
+        </is>
+      </c>
+      <c r="L40" s="21" t="inlineStr">
+        <is>
+          <t>@10</t>
+        </is>
+      </c>
+      <c r="M40" s="21" t="inlineStr">
+        <is>
+          <t>@100</t>
+        </is>
+      </c>
+      <c r="N40" s="21" t="inlineStr">
+        <is>
+          <t>@1,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="C41" s="27" t="inlineStr">
+        <is>
+          <t>E-paper version, 150 mAh ('Cost by batch' total)</t>
+        </is>
+      </c>
+      <c r="L41" s="30">
+        <f>'Cost by batch'!L23</f>
+        <v/>
+      </c>
+      <c r="M41" s="30">
+        <f>'Cost by batch'!M23</f>
+        <v/>
+      </c>
+      <c r="N41" s="30">
+        <f>'Cost by batch'!N23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="C42" s="31" t="inlineStr">
+        <is>
+          <t>LCD version, 150 mAh (this sheet's total)</t>
+        </is>
+      </c>
+      <c r="L42" s="32">
+        <f>L23</f>
+        <v/>
+      </c>
+      <c r="M42" s="32">
+        <f>M23</f>
+        <v/>
+      </c>
+      <c r="N42" s="32">
+        <f>N23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" s="27" t="inlineStr">
+        <is>
+          <t>Difference LCD − e-paper</t>
+        </is>
+      </c>
+      <c r="L43" s="30">
+        <f>L42-L41</f>
+        <v/>
+      </c>
+      <c r="M43" s="30">
+        <f>M42-M41</f>
+        <v/>
+      </c>
+      <c r="N43" s="30">
+        <f>N42-N41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="C44" s="27" t="inlineStr">
+        <is>
+          <t>1,200-1,500 mAh cell (@10 Adafruit #258 1,200 mAh; @100+ Alibaba 504060 ~1,500 mAh)</t>
+        </is>
+      </c>
+      <c r="L44" s="28" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="M44" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="N44" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>Adafruit #258 $9.95 (enclosure/final_assembly/battery_upgrade.md); Alibaba 504060 ~$3-5 at MOQ (estimate). Needs UN38.3 in the seller's name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="C45" s="27" t="inlineStr">
+        <is>
+          <t>Its dangerous-goods freight surcharge</t>
+        </is>
+      </c>
+      <c r="L45" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="28" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="N45" s="28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>Estimate (~5.5 Wh, heavier cell).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="C46" s="27" t="inlineStr">
+        <is>
+          <t>Longer JST-PH lead / extension (~150 mm)</t>
+        </is>
+      </c>
+      <c r="L46" s="28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M46" s="28" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N46" s="28" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>Estimate. Board: R2 20 k → 4.7 k for a ~3 h charge (no cost change).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" s="27" t="inlineStr">
+        <is>
+          <t>Battery change per unit incl. overage %</t>
+        </is>
+      </c>
+      <c r="L47" s="30">
+        <f>(L44+L45+L46-I9-I10)*(1+I19)</f>
+        <v/>
+      </c>
+      <c r="M47" s="30">
+        <f>(M44+M45+M46-J9-J10)*(1+J19)</f>
+        <v/>
+      </c>
+      <c r="N47" s="30">
+        <f>(N44+N45+N46-K9-K10)*(1+K19)</f>
+        <v/>
+      </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>(big cell + its DG + lead − 150 mAh cell − its DG) × (1 + overage %).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" s="27" t="inlineStr">
+        <is>
+          <t>E-paper version, 1,200-1,500 mAh</t>
+        </is>
+      </c>
+      <c r="L48" s="30">
+        <f>L41+L47</f>
+        <v/>
+      </c>
+      <c r="M48" s="30">
+        <f>M41+M47</f>
+        <v/>
+      </c>
+      <c r="N48" s="30">
+        <f>N41+N47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="C49" s="31" t="inlineStr">
+        <is>
+          <t>LCD version, 1,200-1,500 mAh (long-term target, custom or roomy knockoff shell)</t>
+        </is>
+      </c>
+      <c r="L49" s="32">
+        <f>L42+L47</f>
+        <v/>
+      </c>
+      <c r="M49" s="32">
+        <f>M42+M47</f>
+        <v/>
+      </c>
+      <c r="N49" s="32">
+        <f>N42+N47</f>
+        <v/>
+      </c>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t>Fits the custom drop-in shell pocket (70 × 41 × 5.4 mm). In a knockoff only if K-D7/K-S5 show room (KNOCKOFF_SHELL_PLAN.md).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId12"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4334,7 +6334,7 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>PCB + Standard PCBA, v14 files (hardware/fab)</t>
+          <t>PCB + Standard PCBA, v14 files (hardware/fab); v15-LCD files hardware/fab_v15_lcd/ (verified ORDER, review 14)</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -4428,6 +6428,366 @@
         </is>
       </c>
       <c r="L40" s="7" t="inlineStr">
+        <is>
+          <t>100 / 1,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>LCD 1.9" 170x320 (v15)</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Adafruit (US)</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Adafruit</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>1.9" 320x170 IPS TFT breakout, ST7789 (#5394); panel inside = our 30-pin panel</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>open listing</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>$17.50 / $15.75 (10) / $14.00 (100)</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>In stock, 2-3 days</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>Breakout does not fit; peel the panel off</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>Optional FALLBACK only (the ER-TFT019-1 replaced it on 2026-10-08). Same 30-pin glass inside; take it off the breakout.</t>
+        </is>
+      </c>
+      <c r="L41" s="7" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>LCD 1.9" 170x320 (v15)</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Jessinie Store</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>1.9 inch IPS bare screen 30Pin plug-in, ST7789 (FPC NFP190B-21AF / -21A)</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>open listing</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>$2.82 (sale; list $3.76) + $5.27 shipping [S11]</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>Delivery Oct 17-24 (seen 10/8)</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>Choice/standard</t>
+        </is>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>Superseded by Alibaba Goldenmorning / ZJY for bulk. If bought: 30Pin variant, ST7789 (NOT the DJ9853 clone); diode test; tail 36.6 mm.</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>not planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>LCD 1.9" 170x320 (v15)</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Manufacturer</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>NoseDisplay</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>ND019TSN170320-A01 1.9" 170x320 IPS, ST7789P3, 30-pin; custom FPC length offered</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>open listing</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>RFQ [S12]</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>Samples on request</t>
+        </is>
+      </c>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>Outline 25.10 x 49.30 x 2.10 mm (0.1 mm over the 2.0 limit); pins 1-24 as TFT1901; ask for an 18-20 mm tail and pins 25-30.</t>
+        </is>
+      </c>
+      <c r="L43" s="7" t="inlineStr">
+        <is>
+          <t>100 / 1,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>LCD 1.9" 170x320 (v15)</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Manufacturer</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>BuyDisplay / East Rising</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>ER-TFT019-1 1.9" 170x320 IPS, ST7789P3, 4-SPI/8080, no-touch version; custom FPC service</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>open listing</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>~$6-7 (1) / $6.22 (10) / $5.71 (100) [S13]</t>
+        </is>
+      </c>
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>In stock</t>
+        </is>
+      </c>
+      <c r="J44" s="7" t="inlineStr">
+        <is>
+          <t>Shipping per order (check at checkout)</t>
+        </is>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>CHOSEN prototype panel (review 14): datasheet rev 2.0 checked pin for pin vs J5; 25.80 x 49.72 x 1.43 mm, tail 36.6 ± 0.3 mm, VLED 2.8-3.2 V @ 60 mA (R23 = 15 Ω). The ER-CON30HT-1 socket is NOT needed.</t>
+        </is>
+      </c>
+      <c r="L44" s="7" t="inlineStr">
+        <is>
+          <t>prototypes (3) / 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>LCD 1.9" 170x320 (v15)</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Shenzhen Goldenmorning Electronic Co., Ltd.</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>T190X7-C30-01 1.9" 170x320 IPS, ST7789P3, 30-pin (pin table verified)</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>open listing</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>$1.85-2.50, excl. shipping [S15]</t>
+        </is>
+      </c>
+      <c r="I45" s="7" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>Recommended SAMPLE. Ask for the plastic-frame ~1.4 mm build (datasheet shows a 2.11 mm metal frame, too thick).</t>
+        </is>
+      </c>
+      <c r="L45" s="7" t="inlineStr">
+        <is>
+          <t>samples / 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>LCD 1.9" 170x320 (v15)</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Zhengzhou Zhongjingyuan Electronic Technology (ZJY)</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>1.9" 170x320 30-pin TFT, ST7789V3</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>open listing</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>$2.50 @100 / $2.30 @1,000 [S15]</t>
+        </is>
+      </c>
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="J46" s="7" t="inlineStr">
+        <is>
+          <t>Express / sea</t>
+        </is>
+      </c>
+      <c r="K46" s="7" t="inlineStr">
+        <is>
+          <t>Recommended BULK. Confirm the drawing and pin table first (pin 7 SCL, 8 RS, 20 LEDA, 21-24 LEDK); ask about an 18-20 mm FPC tail.</t>
+        </is>
+      </c>
+      <c r="L46" s="7" t="inlineStr">
         <is>
           <t>100 / 1,000</t>
         </is>
@@ -4476,140 +6836,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId43"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Supplier message templates (paste into Alibaba chat / email; replace [brackets])</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="18" t="inlineStr">
-        <is>
-          <t>For</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>Message</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>Any supplier: first contact</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Hi, I'm developing a small handheld electronics product in the USA. I'd like 2 samples of [item / listing link] first, then possibly [100] and later [1,000] pcs. Please send: (1) price tiers for 10 / 100 / 1,000 / 3,000 pcs, (2) sample price + DHL shipping to [ZIP] USA, (3) lead time for each quantity, (4) datasheet / drawing, (5) whether you can use Trade Assurance. Thank you!</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>Knockoff calculator (shell)</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Hi, I'm interested in your 991ES PLUS scientific calculator [link]. Before ordering 2 samples, please send: (1) photos of the inside with the circuit board removed, (2) a photo of the rubber key-mat contact side, (3) the model number and mould number, and confirmation future orders use the SAME mould, (4) outer size and screw positions, (5) price for 10 / 100 / 1,000 pcs, plain version with NO brand logo printed. Can you supply the shell + key mat + window + screws + slide cover without the PCB and battery?</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>OV5640 AF camera</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Hi, I need an OV5640 autofocus DVP module with a 24-pin 0.5 mm FPC, same pinout as the Seeed 'OV5640 for XIAO ESP32S3 Sense'. Please send the FPC pinout drawing, the FPC length and contact side, lens FOV, and AF driver. Can you make the FPC [xx] mm long? Price for 2 samples, 100 and 1,000 pcs, and lead time please.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>E-paper (Good Display)</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Hi Good Display team, I'm using the GDEY0213B74 (2.13" B/W, SSD1680, 24-pin FPC) in a handheld product. Please quote 10, 100 and 1,000 pcs of the bare panel, with lead time and DHL shipping to [ZIP] USA. Please also confirm the current datasheet version and that the FPC pin order is unchanged. Is there an MOQ?</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>LiPo battery</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Hi, I need a 3.7 V LiPo, about 150 mAh, about 26 x 20 x 3.8 mm and at most 33.5 x 20.7 x 3.8 mm INCLUDING the protection board, with a JST-PH 2.0 plug, red wire = + (photo please, same polarity as Adafruit #1317), lead length [xx] mm. Please send: UN38.3 test summary, MSDS/SDS, IEC 62133 (CB) report for THIS model in your company name, the cell model (e.g. 382026/402025), price for 2 samples / 100 / 1,000, and how you ship batteries to the USA (UN3481).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>Magnetic connector + cable</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Hi, I need a 4-pin magnetic pogo connector pair, ~2.54 mm pitch, plus a matching USB-A (or USB-C) magnetic cable, 60 cm. The board half is right-angle (or board-edge SMT). Please send a dimensioned drawing with magnet polarity. Pin order on the cable plug, N to S: GND, D+, D-, VBUS (USB data must work, not only charging). Price for 2 sample sets / 100 / 1,000 and lead time please. Can you customise pin order and cable length?</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>Packaging</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Hi, please quote a printed box with a die-cut foam/EVA insert for a calculator ([L x W x H] mm) plus a USB cable. Quantities 100 and 1,000, 1 colour print outside, and the price of a printed sample. Please send the die-line template, and quote a small folded manual (A6, 8 pages, B/W) too.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>Follow-up / negotiation</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Thank you for the quote. Samples arrived and passed. For the [100] pcs order: can you match [$x], keep the same materials/revision as the samples, and send photos of the finished goods before shipping? Please confirm in the PI that the product matches the approved sample.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4620,7 +6853,152 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Supplier message templates (paste into Alibaba chat / email; replace [brackets])</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>For</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>Any supplier: first contact</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Hi, I'm developing a small handheld electronics product in the USA. I'd like 2 samples of [item / listing link] first, then possibly [100] and later [1,000] pcs. Please send: (1) price tiers for 10 / 100 / 1,000 / 3,000 pcs, (2) sample price + DHL shipping to [ZIP] USA, (3) lead time for each quantity, (4) datasheet / drawing, (5) whether you can use Trade Assurance. Thank you!</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>Knockoff calculator (shell)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Hi, I'm interested in your 991ES PLUS scientific calculator [link]. Before ordering 2 samples, please send: (1) photos of the inside with the circuit board removed, (2) a photo of the rubber key-mat contact side, (3) the model number and mould number, and confirmation future orders use the SAME mould, (4) outer size and screw positions, (5) price for 10 / 100 / 1,000 pcs, plain version with NO brand logo printed. Can you supply the shell + key mat + window + screws + slide cover without the PCB and battery?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>OV5640 AF camera</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Hi, I need an OV5640 autofocus DVP module with a 24-pin 0.5 mm FPC, same pinout as the Seeed 'OV5640 for XIAO ESP32S3 Sense'. Please send the FPC pinout drawing, the FPC length and contact side, lens FOV, and AF driver. Can you make the FPC [xx] mm long? Price for 2 samples, 100 and 1,000 pcs, and lead time please.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>E-paper (Good Display)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Hi Good Display team, I'm using the GDEY0213B74 (2.13" B/W, SSD1680, 24-pin FPC) in a handheld product. Please quote 10, 100 and 1,000 pcs of the bare panel, with lead time and DHL shipping to [ZIP] USA. Please also confirm the current datasheet version and that the FPC pin order is unchanged. Is there an MOQ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>LiPo battery</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Hi, I need a 3.7 V LiPo, about 150 mAh, about 26 x 20 x 3.8 mm and at most 33.5 x 20.7 x 3.8 mm INCLUDING the protection board, with a JST-PH 2.0 plug, red wire = + (photo please, same polarity as Adafruit #1317), lead length [xx] mm. Please send: UN38.3 test summary, MSDS/SDS, IEC 62133 (CB) report for THIS model in your company name, the cell model (e.g. 382026/402025), price for 2 samples / 100 / 1,000, and how you ship batteries to the USA (UN3481).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Magnetic connector + cable</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Hi, I need a 4-pin magnetic pogo connector pair, ~2.54 mm pitch, plus a matching USB-A (or USB-C) magnetic cable, 60 cm. The board half is right-angle (or board-edge SMT). Please send a dimensioned drawing with magnet polarity. Pin order on the cable plug, N to S: GND, D+, D-, VBUS (USB data must work, not only charging). Price for 2 sample sets / 100 / 1,000 and lead time please. Can you customise pin order and cable length?</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Hi, please quote a printed box with a die-cut foam/EVA insert for a calculator ([L x W x H] mm) plus a USB cable. Quantities 100 and 1,000, 1 colour print outside, and the price of a printed sample. Please send the die-line template, and quote a small folded manual (A6, 8 pages, B/W) too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>Follow-up / negotiation</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Thank you for the quote. Samples arrived and passed. For the [100] pcs order: can you match [$x], keep the same materials/revision as the samples, and send photos of the finished goods before shipping? Please confirm in the PI that the product matches the approved sample.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>LCD 1.9" panel (v15)</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>Hi [supplier] team, I'm using a 1.9" 170x320 IPS TFT with an ST7789 controller and a 30-pin 0.5 mm FPC (same as BuyDisplay ER-TFT019-1 / TFT1901 / N190-1732TBWPG01, the LilyGO T-Display-S3 panel) in a handheld product. Please quote 10, 100 and 1,000 pcs, with lead time and DHL shipping to [ZIP] USA. Please send the drawing and datasheet, confirm the controller is ST7789 (not a clone), the pin order (pin 7 SCL, 8 RS, 20 LEDA, 21-24 LEDK), the FPC tail length, and whether you can make the FPC tail 18-20 mm long (MOQ and price). Please quote the plastic-frame (about 1.4 mm thick) build, not the 2.1 mm metal frame. Is there an MOQ?</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4964,18 +7342,43 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>LCD (v15)</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Diode test on the first panels of every batch: LED drop (~2.6 V) between finger 20 and fingers 21-24 (ER-TFT019-1: cathode on 22); check the tail length (36.6 ± 0.3 mm), the frame thickness (plastic ~1.4 mm) and the controller (ST7789).</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>J5 is numbered for one tail direction (verification/13 S1, confirmed on the ER-TFT019-1 drawing in verification/14); clone controllers need other init code.</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>LED fingers in the TOP half of J5; colour bars + backlight sweep pass in the self-test.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5180,15 +7583,100 @@
     <row r="13">
       <c r="A13" s="21" t="inlineStr">
         <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>AliExpress 1.9" 30Pin ST7789 bare panel $2.82 + $5.27 shipping (seen 2026-10-08; hardware/LCD_PANEL_OPTIONS.md row B)</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>hardware/LCD_PANEL_OPTIONS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>NoseDisplay ND019TSN170320-A01 (custom FPC length offered)</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>https://www.nosedisplay.com/products/1-9-inch-tft-display-170x320-resolution-spi-interface-st7789p3-controller-ips-screen/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>BuyDisplay ER-TFT019-1 1.9" 170x320 ST7789P3 (datasheet rev 2.0 checked 2026-10-08, verification/14): ~$6-7, $6.22 @10, $5.71 @100</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>https://www.buydisplay.com/full-viewing-angle-spi-1-9-inch-ips-tft-lcd-display-panel-170x320-st7789</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>Adafruit #5394 1.9" 320x170 IPS breakout $17.50 / #258 1,200 mAh LiPo $9.95</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>https://www.adafruit.com/product/5394</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>Alibaba LCD search 2026-10-08 (Goldenmorning sample $1.85-2.50; ZJY $2.50 @100 / $2.30 @1,000): hardware/production/lcd_suppliers.json</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>https://www.alibaba.com/product-detail/1-9-Inch-170x320-30-PIN_1600647344150.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>Alibaba product pages returned a CAPTCHA to automated reading on 2026-10-05; numbers are from search-index snippets and must be confirmed by RFQ.</t>
         </is>
       </c>
-      <c r="C13" s="22" t="inlineStr"/>
+      <c r="C18" s="22" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Docs: propagate corrected zone datums, battery tape strip-2 margin, key-mat orientation, TW302030 to older docs and sheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Claude outputs/Alibaba_Bulk_Sourcing.xlsx
+++ b/Claude outputs/Alibaba_Bulk_Sourcing.xlsx
@@ -1084,7 +1084,7 @@
       </c>
       <c r="R9" s="12" t="inlineStr">
         <is>
-          <t>Adafruit #1317 $5.95 [S8] (switched from the 100 mAh #1570 on 2026-10-06; same price). Alibaba 401230 listings $0.56-1.60 [S6] are 100 mAh references (401230 is 4.0 x 12 x 30: too thick and wide); ask for a ~150 mAh cell in 26 x 20 x 3.8. @100/@1,000 include PH lead + PCM (estimate).</t>
+          <t>Adafruit #1317 $5.95 [S8] (switched from the 100 mAh #1570 on 2026-10-06; same price). Alibaba 401230 listings $0.56-1.60 [S6] are 100 mAh references (401230 is 4.0 x 12 x 30: too thick and wide); ask for a ~150 mAh cell in 26 x 20 x 3.8. @100/@1,000 include PH lead + PCM (estimate). Named bulk candidate (2026-10-10): Taiwoo TW302030, 140 mAh, 30 × 20 × 3.0; fits the fx-115ES spot in CAD when placed 1 mm left of the #1317 position ('Supplier options' row 49); price not yet quoted, so the estimates stand.</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6912,6 +6912,66 @@
         </is>
       </c>
       <c r="L48" s="7" t="inlineStr">
+        <is>
+          <t>100 / 1,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>LiPo ~150 mAh</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Alibaba</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Taiwoo (TW302030 listing)</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>Taiwoo TW302030 LiPo 3.7 V 140 mAh, L 30 (+2/−0.5) × W 20 ± 0.5 × T 3.0 ± 0.3 mm incl. PCB; connector 1.0 / 1.25 / 2.0 mm; PCM customised (3.0 V cut-off available)</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>no link yet</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>Ask (not price-checked)</t>
+        </is>
+      </c>
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="J49" s="7" t="inlineStr">
+        <is>
+          <t>DG (UN3481); ask for UN38.3 + MSDS</t>
+        </is>
+      </c>
+      <c r="K49" s="7" t="inlineStr">
+        <is>
+          <t>CAD fit-checked 2026-10-10 on v14 and v15 (hardware/enclosure/final_assembly/variant_battery_tw302030/results.json): FITS when placed 1 mm LEFT of the #1317 position (left edge ~1.7 mm from the corner post, top edge 0.8 mm from the lip; a cell over ~20.3 mm wide goes right up to the lip). Ask for: PCM included; JST-PH 2.0 2-pin, red (+) on pin 2, black on pin 1 (photo); leads 50–80 mm leaving the short (lead) end; UN38.3 + MSDS in the seller's name. Meter the polarity of every sample.</t>
+        </is>
+      </c>
+      <c r="L49" s="7" t="inlineStr">
         <is>
           <t>100 / 1,000</t>
         </is>

</xml_diff>